<commit_message>
Add Exercise5B to week-01
</commit_message>
<xml_diff>
--- a/week-01/Ex5B_Robera Coffee Shop Survey.xlsx
+++ b/week-01/Ex5B_Robera Coffee Shop Survey.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yearuptemp-my.sharepoint.com/personal/hmerawi_my_yearupunited_org/Documents/Desktop/Documents/DataAnalytics/week-01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{0912672F-9CF6-45F2-A2AE-F6A78B0C8CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{105EE3FC-5630-4AE7-B1EE-076B53D0673A}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="14_{EB2F1637-35DB-4B28-8900-2541F7C7D162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42411D9A-8989-42BE-9242-441D14872A4E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="36">
   <si>
     <t>Id</t>
   </si>
@@ -187,10 +187,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -206,7 +205,22 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -221,39 +235,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="mm:ss:"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="mm:ss:"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -266,13 +247,31 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="mm:ss:"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="mm:ss:"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -301,7 +300,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Robera Coffee Shop Survey.xlsx]Sheet2!PivotTable1</c:name>
+    <c:name>[Ex5B_Robera Coffee Shop Survey.xlsx]Sheet2!PivotTable1</c:name>
     <c:fmtId val="0"/>
   </c:pivotSource>
   <c:chart>
@@ -422,7 +421,7 @@
         <c:idx val="1"/>
         <c:spPr>
           <a:solidFill>
-            <a:schemeClr val="accent3"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln>
             <a:noFill/>
@@ -528,7 +527,7 @@
         <c:idx val="3"/>
         <c:spPr>
           <a:solidFill>
-            <a:schemeClr val="accent2"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln>
             <a:noFill/>
@@ -581,7 +580,7 @@
         <c:idx val="4"/>
         <c:spPr>
           <a:solidFill>
-            <a:schemeClr val="accent4"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln>
             <a:noFill/>
@@ -978,6 +977,540 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[Ex5B_Robera Coffee Shop Survey.xlsx]Sheet2!PivotTable2</c:name>
+    <c:fmtId val="2"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Visit Frequency</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$B$16</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$17:$A$20</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2-3 times a week</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Daily</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Weekly</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$17:$B$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-802C-43F0-A3A2-4253690F8622}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1947440448"/>
+        <c:axId val="1947441888"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1947440448"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1947441888"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1947441888"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1947440448"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1018,7 +1551,550 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -1559,6 +2635,44 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7D526C81-4501-4EA3-AA07-B94A3668C6FA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1600,7 +2714,11 @@
       </sharedItems>
     </cacheField>
     <cacheField name="How often do you visit us?" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="3">
+        <s v="Weekly"/>
+        <s v="2-3 times a week"/>
+        <s v="Daily"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="What reward would make you come back more often?" numFmtId="0">
       <sharedItems/>
@@ -1631,7 +2749,7 @@
     <m/>
     <n v="3"/>
     <x v="0"/>
-    <s v="Weekly"/>
+    <x v="0"/>
     <s v="Free size upgrade"/>
     <n v="3"/>
     <s v="sakura drinks"/>
@@ -1645,7 +2763,7 @@
     <m/>
     <n v="5"/>
     <x v="1"/>
-    <s v="2-3 times a week"/>
+    <x v="1"/>
     <s v="Free drink after 6 purchases"/>
     <n v="4"/>
     <s v="Caramel Granita :)"/>
@@ -1659,7 +2777,7 @@
     <m/>
     <n v="5"/>
     <x v="0"/>
-    <s v="Weekly"/>
+    <x v="0"/>
     <s v="Free size upgrade"/>
     <n v="5"/>
     <s v="lavender earl grey"/>
@@ -1673,7 +2791,7 @@
     <m/>
     <n v="5"/>
     <x v="1"/>
-    <s v="Daily"/>
+    <x v="2"/>
     <s v="15% off for students"/>
     <n v="5"/>
     <s v="Cheesecake "/>
@@ -1687,7 +2805,7 @@
     <m/>
     <n v="1"/>
     <x v="1"/>
-    <s v="Daily"/>
+    <x v="2"/>
     <s v="Free drink after 6 purchases"/>
     <n v="1"/>
     <s v="close store"/>
@@ -1701,7 +2819,7 @@
     <m/>
     <n v="4"/>
     <x v="0"/>
-    <s v="2-3 times a week"/>
+    <x v="1"/>
     <s v="Free size upgrade"/>
     <n v="4"/>
     <s v="Pineapple tea "/>
@@ -1715,7 +2833,7 @@
     <m/>
     <n v="4"/>
     <x v="1"/>
-    <s v="Weekly"/>
+    <x v="0"/>
     <s v="15% off for students"/>
     <n v="5"/>
     <s v="I would like to see a reposado espresso."/>
@@ -1729,7 +2847,7 @@
     <m/>
     <n v="3"/>
     <x v="2"/>
-    <s v="Weekly"/>
+    <x v="0"/>
     <s v="Free drink after 6 purchases"/>
     <n v="4"/>
     <s v="no"/>
@@ -1743,7 +2861,7 @@
     <m/>
     <n v="2"/>
     <x v="3"/>
-    <s v="2-3 times a week"/>
+    <x v="1"/>
     <s v="15% off for students"/>
     <n v="3"/>
     <s v="Pomegranate "/>
@@ -1757,7 +2875,7 @@
     <m/>
     <n v="5"/>
     <x v="3"/>
-    <s v="2-3 times a week"/>
+    <x v="1"/>
     <s v="Free drink after 6 purchases"/>
     <n v="5"/>
     <s v="the place could be cleaner. thank you"/>
@@ -1766,7 +2884,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4001D0D-F01F-4B40-853B-0F9108C64AC6}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4001D0D-F01F-4B40-853B-0F9108C64AC6}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="A1:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
@@ -1892,85 +3010,164 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7F84985B-BEC5-4214-8CAD-CF6749EAC0D8}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="A16:B20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Email" fld="4" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="2">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:L12" totalsRowCount="1">
   <autoFilter ref="A1:L11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="15" totalsRowDxfId="11">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="23" totalsRowDxfId="22">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="id"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="14" totalsRowDxfId="10">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="21" totalsRowDxfId="20">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="startDate"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="13" totalsRowDxfId="9">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="19" totalsRowDxfId="18">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="submitDate"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{389A4EA4-BDB0-47CD-AE50-2414F84177D6}" name="Time to Complete" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="8">
+    <tableColumn id="12" xr3:uid="{389A4EA4-BDB0-47CD-AE50-2414F84177D6}" name="Time to Complete" totalsRowFunction="custom" dataDxfId="17" totalsRowDxfId="16">
       <calculatedColumnFormula>C2-B2</calculatedColumnFormula>
       <totalsRowFormula>AVERAGE(D2:D11)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="23" totalsRowDxfId="7">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="15" totalsRowDxfId="14">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="responder"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name Rating" dataDxfId="22" totalsRowDxfId="6">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name Rating" dataDxfId="13" totalsRowDxfId="12">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="responderName"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="How would you rate the taste of your coffee today?" dataDxfId="21" totalsRowDxfId="5">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="How would you rate the taste of your coffee today?" dataDxfId="11" totalsRowDxfId="10">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rbf1c3e46fc2e427d876a483f178d661f"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="What is your go-to drink?" dataDxfId="20" totalsRowDxfId="4">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="What is your go-to drink?" dataDxfId="9" totalsRowDxfId="8">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rf0847a93cc444bed930bfd60637cdae7"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="How often do you visit us?" dataDxfId="19" totalsRowDxfId="3">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="How often do you visit us?" dataDxfId="7" totalsRowDxfId="6">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r930daa4a95e344889dcac03e376f28fb"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="What reward would make you come back more often?" dataDxfId="18" totalsRowDxfId="2">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="What reward would make you come back more often?" dataDxfId="5" totalsRowDxfId="4">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r0343a9f1efbd4e9fb6f832a90c83e997"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="How is our Wi-Fi speed and seating comfort?" dataDxfId="17" totalsRowDxfId="1">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="How is our Wi-Fi speed and seating comfort?" dataDxfId="3" totalsRowDxfId="2">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r6dc412affb2d4693b4fda0cbed1ca220"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Any suggestions for new seasonal flavors you'd like to see?" dataDxfId="16" totalsRowDxfId="0">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Any suggestions for new seasonal flavors you'd like to see?" dataDxfId="1" totalsRowDxfId="0">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r89deacc5860b4e3aa5832304eddf2d5a"/>
@@ -2300,9 +3497,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.77734375" customWidth="1"/>
-    <col min="2" max="2" width="21.77734375" style="3" customWidth="1"/>
+    <col min="2" max="2" width="21.77734375" style="2" customWidth="1"/>
     <col min="3" max="3" width="21.77734375" customWidth="1"/>
-    <col min="4" max="4" width="21.77734375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="21.77734375" style="3" customWidth="1"/>
     <col min="5" max="16" width="21.77734375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2310,13 +3507,13 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>31</v>
       </c>
       <c r="E1" t="s">
@@ -2348,13 +3545,13 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>46120.374120370368</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>46120.374664351853</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <f t="shared" ref="D2:D11" si="0">C2-B2</f>
         <v>5.4398148495238274E-4</v>
       </c>
@@ -2384,13 +3581,13 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>46120.410879629628</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>46120.411157407405</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <f t="shared" si="0"/>
         <v>2.7777777722803876E-4</v>
       </c>
@@ -2420,13 +3617,13 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>46120.56391203704</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>46120.564340277779</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <f t="shared" si="0"/>
         <v>4.2824073898373172E-4</v>
       </c>
@@ -2456,13 +3653,13 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>46120.573888888888</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>46120.574652777781</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <f t="shared" si="0"/>
         <v>7.638888928340748E-4</v>
       </c>
@@ -2492,13 +3689,13 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>46120.613263888888</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>46120.613495370373</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <f t="shared" si="0"/>
         <v>2.3148148466134444E-4</v>
       </c>
@@ -2528,13 +3725,13 @@
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>46120.614166666666</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>46120.615115740744</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <f t="shared" si="0"/>
         <v>9.490740776527673E-4</v>
       </c>
@@ -2564,13 +3761,13 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>46121.481099537035</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>46121.488009259258</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <f t="shared" si="0"/>
         <v>6.9097222221898846E-3</v>
       </c>
@@ -2600,13 +3797,13 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>46121.491122685184</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <v>46121.492303240739</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <f t="shared" si="0"/>
         <v>1.1805555550381541E-3</v>
       </c>
@@ -2636,13 +3833,13 @@
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>46121.494745370372</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <v>46121.494803240741</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <f t="shared" si="0"/>
         <v>5.7870369346346706E-5</v>
       </c>
@@ -2672,13 +3869,13 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>46121.536423611098</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>46121.5368171296</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <f t="shared" si="0"/>
         <v>3.9351850136881694E-4</v>
       </c>
@@ -2706,19 +3903,16 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="4">
+      <c r="C12" s="2"/>
+      <c r="D12" s="3">
         <f>AVERAGE(D2:D11)</f>
         <v>1.1736111104255543E-3</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="2"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-      <c r="K12" s="2"/>
       <c r="L12" s="1"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -2752,7 +3946,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{594618AD-0E14-404A-8C61-258BBF935496}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
@@ -2760,7 +3954,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B1" t="s">
@@ -2768,47 +3962,87 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>